<commit_message>
Auto update Pengadaan 2026-10-23 08:09:48
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-23).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-23).xlsx
@@ -1004,35 +1004,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1154,35 +1146,27 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>3839600910</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -1308,13 +1292,13 @@
         <v>93</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1145584728</v>
+        <v>1148350728</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>61019294</v>
+        <v>63785294</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>7</v>
@@ -1339,22 +1323,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>414639535</v>
+        <v>403884747</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>78869208</v>
+        <v>128214258</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1373,22 +1357,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>963345953</v>
+        <v>961842399</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>137583844</v>
+        <v>136080290</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>116218702</v>
+        <v>1520271914</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>109</v>
@@ -1407,22 +1391,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>338050900</v>
+        <v>3037348900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1444,13 +1428,13 @@
         <v>135</v>
       </c>
       <c r="D27" s="10" t="n">
-        <v>1128213815</v>
+        <v>1128233165</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>37</v>
       </c>
       <c r="F27" s="10" t="n">
-        <v>303814298</v>
+        <v>303833648</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>37</v>
@@ -1478,13 +1462,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>900575817</v>
+        <v>890948817</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>38508000</v>
+        <v>28881000</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1</v>
@@ -1512,13 +1496,13 @@
         <v>186</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>2526072363</v>
+        <v>2516568210</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>58</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>58</v>
@@ -1543,22 +1527,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>90550292</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>86612607</v>
+        <v>236612607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>44</v>
@@ -1580,13 +1564,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>283301771</v>
+        <v>283157746</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>30262050</v>
+        <v>30118025</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1614,13 +1598,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>767894130</v>
+        <v>764274671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1648,13 +1632,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>366634933</v>
+        <v>278301799</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1716,13 +1700,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>463972148</v>
+        <v>463836830</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1750,13 +1734,13 @@
         <v>76</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>761771973</v>
+        <v>761250273</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>13</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>334343818</v>
+        <v>333822118</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>13</v>
@@ -1781,28 +1765,28 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>1235454791</v>
+        <v>854862891</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>412496502</v>
+        <v>81094602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>402113040</v>
+        <v>1296895670</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>822958289</v>
+        <v>773768289</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -1818,13 +1802,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>384332451</v>
+        <v>382731831</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>12</v>
@@ -1849,22 +1833,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>1337901275</v>
+        <v>1312371275</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>391109425</v>
+        <v>365579425</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>387344886</v>
+        <v>427421436</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>86</v>
@@ -1988,13 +1972,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>708077545</v>
+        <v>727698127</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2019,22 +2003,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>340998868</v>
+        <v>270482868</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>151137140</v>
+        <v>80621140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>18</v>
@@ -2103,22 +2087,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1071589309</v>
+        <v>1120241719</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>161</v>
@@ -2224,13 +2208,13 @@
         <v>102</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>608286476</v>
+        <v>606361476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>238522198</v>
+        <v>236597198</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>18</v>
@@ -2339,30 +2323,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3132,13 +3110,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>330321582</v>
+        <v>323431257</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3163,22 +3141,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3284,7 +3262,7 @@
         <v>113</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>1433154546</v>
+        <v>1398754546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3302,7 +3280,7 @@
         <v>95</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>1013280360</v>
+        <v>978880360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3318,13 +3296,13 @@
         <v>145</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1492289470</v>
+        <v>1484655470</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>24</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>207985114</v>
+        <v>200351114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>24</v>
@@ -3347,28 +3325,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4034</v>
+        <v>4086</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>35200200506</v>
+        <v>34618027872</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>507</v>
+        <v>558</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>7807108387</v>
+        <v>7308525753</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>507</v>
+        <v>558</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6828104524.6</v>
+        <v>20178290216.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3527</v>
+        <v>3528</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27393092119</v>
+        <v>27309502119</v>
       </c>
     </row>
   </sheetData>
@@ -3789,13 +3767,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4225,45 +4203,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4295,29 +4257,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>111200910</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>111200910</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -4540,34 +4518,50 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>323734637</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="K24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <v>49345050</v>
+        <v>268961631</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4586,34 +4580,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1848714675</v>
+        <v>1679001832</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>1225542538</v>
+        <v>1055829695</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>323493965</v>
+        <v>258068473</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>7</v>
@@ -4832,28 +4826,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
@@ -4885,13 +4879,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>477133090</v>
+        <v>490395090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5085,13 +5079,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>1694840343</v>
+        <v>1667542131</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>913021368</v>
+        <v>885723156</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5135,13 +5129,13 @@
         <v>39</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>5044312982</v>
+        <v>5043896732</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>36</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>36</v>
@@ -5182,40 +5176,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>3419825552</v>
+        <v>2771677052</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>1839090451</v>
+        <v>1376941951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1791219523</v>
+        <v>1333233523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1581713573</v>
+        <v>1123727573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>713727983</v>
+        <v>366519983</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N37" s="10" t="n">
-        <v>1580735101</v>
+        <v>1394735101</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5290,28 +5284,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>4380291888</v>
+        <v>4127193593</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>2674384586</v>
+        <v>2421286291</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2613571243</v>
+        <v>2388524693</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2438894693</v>
+        <v>2253924693</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -5568,28 +5562,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>547117650</v>
+        <v>475135300</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>2</v>
@@ -5684,28 +5678,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>932380105</v>
+        <v>716222170</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
@@ -6028,34 +6022,50 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>660566066</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>340582172</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="K52" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="L52" s="9" t="n">
-        <v>65401200</v>
+        <v>319983894</v>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M52" s="7" t="n">
         <v>4</v>
@@ -7197,13 +7207,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>423288615</v>
+        <v>392285593</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7464,28 +7474,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>3401653729</v>
+        <v>3551653729</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>564698247</v>
+        <v>714698247</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -7512,40 +7522,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>904</v>
+        <v>886</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>106727527526</v>
+        <v>104999095441</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>66296798386</v>
+        <v>64754366301</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64159073617.41</v>
+        <v>63162329768.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>369</v>
+        <v>353</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>45455029518.03</v>
+        <v>44498362219.03</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1611769528</v>
+        <v>1084389786</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>40430729140</v>
+        <v>40244729140</v>
       </c>
     </row>
   </sheetData>
@@ -8347,28 +8357,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8454,29 +8464,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8508,29 +8534,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1081900000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>1081900000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -8566,13 +8608,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8620,7 +8662,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -8666,7 +8708,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8799,40 +8841,40 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>49096492181</v>
+        <v>6460249182</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>47632716881</v>
+        <v>4916473882</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>2945468782</v>
+        <v>1712457037</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N25" s="10" t="n">
-        <v>1463775300</v>
+        <v>1543775300</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -9483,34 +9525,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>5765940896</v>
+        <v>4892340896</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2946694000</v>
+        <v>2073094000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>2509890630</v>
+        <v>2073094000</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>2509890630</v>
-      </c>
-      <c r="K37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="10" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9599,28 +9645,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>3813601480</v>
+        <v>3962367980</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -9826,13 +9872,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11753,28 +11799,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>14398798637</v>
+        <v>7792798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -11965,28 +12011,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>7133067600</v>
+        <v>6783067600</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -12013,40 +12059,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>247</v>
+        <v>215</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>185764047258</v>
+        <v>132047427847</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147457910043</v>
+        <v>93666790632</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71036708305.01001</v>
+        <v>64029064462.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>67370069205</v>
+        <v>60362425362</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4073719266</v>
+        <v>2403910891</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>85</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>38306137215</v>
+        <v>38380637215</v>
       </c>
     </row>
   </sheetData>
@@ -13035,13 +13081,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13085,29 +13131,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>2646500000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>2646500000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -13490,28 +13552,40 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>5399320575</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2699298000</v>
+        <v>2699320575</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -16954,28 +17028,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>278721235553</v>
+        <v>273281535553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147115370800</v>
+        <v>141675670800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>